<commit_message>
feat: add question management module with excel import and filtering capabilities
</commit_message>
<xml_diff>
--- a/frontend/public/Question_Import_Example.xlsx
+++ b/frontend/public/Question_Import_Example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Antigravity\Exam-Generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6013989-106C-45EB-8D41-59034B3AF638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88688688-474D-4423-B42A-02D5D86FF3C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{107AC0EE-0D7C-4BE6-8CAF-E60AC31B08DE}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Câu hỏi</t>
   </si>
@@ -47,60 +47,66 @@
     <t>Đáp án</t>
   </si>
   <si>
-    <t>Yêu cầu khi mở cửa qua bãi vật cản trước tiền duyên phòng ngự của địch
-- Cửa mở phải đúng ý định chiến đấu của người chỉ huy. (1,0đ)
-- Tim cửa mở qua bãi vật cản của ta và cửa mở qua bãi vật cản của địch phải thẳng hướng với nhau. (1,0đ)
-- Cửa mở phải đủ chiều rộng, gọn, sạch. (1,0đ)
-- Phải bình tĩnh, gan dạ, dũng cảm, linh hoạt, xử trí tốt các tình huống xảy ra. (1,0đ)</t>
-  </si>
-  <si>
-    <t>Đồng chí trình bày yêu cầu khi mở cửa qua bãi vật cản trước tiền duyên phòng ngự của địch? (10đx0,4)</t>
-  </si>
-  <si>
-    <t>Đồng chí thực hành vừa nói vừa làm thứ tự các bước bố trí mìn chống bộ binh K-58? (10đx0,5)</t>
-  </si>
-  <si>
-    <t>Các bước bố trí mìn chống bộ binh K-58 
+    <t>Đồng chí nêu khái niệm, nội dung trạng thái sẵn sàng chiến đấu thường xuyên? (10đx0,4)</t>
+  </si>
+  <si>
+    <t>Đồng chí thực hành vừa nói vừa làm động tác gói buộc lượng nổ dài bằng thuốc bánh loại 400g (không có vỏ bọc) trọng lượng 4 kg? (10đx0,5) vừa nói vừa làm thứ tự các bước bố trí mìn chống bộ binh K-58? (10đx0,5)</t>
+  </si>
+  <si>
+    <t>Chọn vị trí bằng phẳng, đặt nẹp lên đà kê, sao cho đầu nẹp cách đà kê 50 ÷ 60cm, hoặc một cánh tay với. (1,0đ)
+- Ngồi theo tư¬ thế vọt tiến chỉ khác chân không thuận đặt lên trên nẹp ở phía trên đà kê. (1,0đ)
+- Xếp thuốc và khí tài ở phía bên tay thuận sao cho dễ lấy. (1,0đ)
+- Rút đầu dây trong của cuộn dây ra và buộc cố định vào đầu nẹp theo nút đầu gà sao cho tạo thành hình tam giác cân để giữ chắc đầu bánh thuốc. (1,0đ)
+- Tay không thuận kéo căng dây, tay thuận xếp thuốc lên trên nẹp. Nếu là bánh thuồc 200g bánh đầu lỗ tra kíp quay lên trên, các bánh tiếp sau lỗ tra kíp quay xuống  d¬ưới. Nếu là bánh thuốc 400g các lỗ tra kíp quay sang hai bên. (1,0đ)
+- Dùng mũi chân không thuận tỳ lên cạnh bánh thuốc cuối cùng, tay thuận chỉnh thuốc. (1,0đ)
+- Chuyển tay cầm cuộn dây sang tay thuận kéo dây cho căng. Dùng ngón cái của tay không thuận giữ dây ở chính giữa mặt bánh thuốc thứ nhất. Tay thuận luồn dây ở d¬ưới nẹp từ bên thuận sang bên không thuận phía dư¬ới tay không thuận. Luồn cuộn dây qua vòng dây và kéo sang bên thuận cho căng, sau đó kéo cuộn dây vào trong lòng. Tay không thuận chỉnh dây sao cho chính giữa mặt bánh thuốc thứ nhất và dây vuông góc với cạnh bánh thuốc. Cứ lần lư¬ợt như¬ vậy tiếp tục lèo dây ở các bánh còn lại đã xếp lên trên nẹp cho tới hết. (2,0đ)
+- Tay thuận kéo căng dây, chân không thuận đặt xuống đất. Tay không thuận tiếp tục lao nẹp lên phía trư¬ớc. Chân không thuận đặt lên nẹp ở phía trên đà kê, chuyển tay cầm cuộn dây sang tay không thuận và tiếp tục gói buộc như trên cho tới khi đủ chiều dài của lượng nổ. (1,0đ)
+- Cố định đầu dây sao cho tạo thành hình tam giác cân, quấn 3÷4 vòng lên trên nẹp và cố định đầu dây lại. (1,0đ)</t>
+  </si>
+  <si>
+    <t>Đồng chí nêu yêu cầu khi bố trí vật cản? (10đx0,4)</t>
+  </si>
+  <si>
+    <t>Yêu cầu khi bố trí vật cản 
+- Bố trí vật cản phải cản được địch nhưng không ảnh hưởng tới hành động của ta, tạo được thế bất ngờ đối với địch. (2,5đ)
+- Bố trí phải kết hợp chặt chẽ giữa địa hình với hoả lực. (2,5đ)
+- Bố trí vật cản phải đạt được hiệu lực chiến đấu cao nhất. (2,5đ)
+- Phải theo kế hoạch thống nhất và theo chỉ thị mệnh lệnh của người chỉ huy từ cấp trung đoàn trở lên. (2,5đ)</t>
+  </si>
+  <si>
+    <t>Đồng chí thực hành vừa nói vừa làm thứ tự các bư¬ớc khi bố trí mìn chống tăng TM-57? (10đx0,5)</t>
+  </si>
+  <si>
+    <t>Thứ tự các bước bố trí mìn chống tăng TM-57 
 a) Công tác chuẩn bị (1,0đ)
-- Mìn và ngòi nổ đảm bảo đủ về số và chất lượng. (0,5đ)
-- Dụng cụ bố trí: Cuốc, xẻng, dao găm, mảnh bao tải, thuốn, túi đựng ngòi nổ. (0,25đ)
-- Vũ khí chiến đấu. (0,25đ)
+- Mìn và ngòi nổ đủ số lượng, đảm bảo chất lượng. (0,5đ)
+- Dụng cụ bố trí: Cuốc, xẻng, túi đựng ngòi nổ; vũ khí chiến đấu. (0,5đ)
 b) Thực hành bố trí (9,0đ)
-- B1: Lấy lớp cỏ nguỵ trang hình bán nguyệt dầy từ 1 2cm. (1,0đ)
-- B2: Đào hố mìn: Đặt mìn ướm thử, đào hố mìn rộng hơn thân mìn; chiều sâu sao cho khi bố trí mìn nơi đất cứng mặt mìn cao hơn mặt đất tự nhiên từ 1-2 cm, đất mềm mặt mìn bằng mặt đất tự nhiên, nơi đất yếu phải gia cố đáy mìn bằng gạch đá, cành cây. (2,0đ)
-- Bước 3: Kiểm tra mìn, ngòi nổ. Lắp chốt chì vào ngòi nổ (nếu chưa có). (2,0)
-- B4: Lắp ngòi nổ vào mìn, vặn nắp bảo hiểm. (1,0đ)
-- B5: Lắp kíp vào thân mìn, vặn nắp bảo hiểm. (1,0đ)
-- B6: Rút chốt an toàn, đặt mìn xuống hố, lấp đất ngụy trang, thu dọn xoá dấu vết, rời khỏi vị trí bố trí (thời gian không quá 5 phút). (2,0đ)</t>
-  </si>
-  <si>
-    <t>Đồng chí cho biết có bao nhiêu quy tắc an toàn khi bố trí mìn,  trình bày quy tắc 1, 2, 3, 4, 5? (10đx0,4)</t>
-  </si>
-  <si>
-    <t>Đồng chí thực hành vừa nói vừa làm thứ tự các bước khi  tháo gỡ mìn chống bộ binh K-58? (10đx0,5)</t>
-  </si>
-  <si>
-    <t>Các bước tháo gỡ mìn chống bộ binh K-58 
-a) Công tác chuẩn bị (1,0đ)
-- Dụng cụ tháo gỡ: Cuốc, xẻng, thuốn, dao găm, mảnh bao tải, túi đựng ngòi nổ. (0,5đ)
-- Vũ khí chiến đấu. (0,5đ)
-b)Thực hành tháo gỡ (9,0đ)
-- Ngồi theo tư thế chiến sỹ, mặt quay về hướng địch. Dùng thuốn kiểm tra xác định vị trí bố trí mìn, trải mảnh bao tải, tiến hành tháo gỡ qua 6 bước (1,0đ)
-- B1: Nhẹ nhàng bới lớp cỏ ngụy trang cho lộ rõ mặt mìn và thành mìn. (1,0đ)
-- B2:  Dùng thuốn kiểm tra xung quanh mìn (nếu cần). (2,0đ)
-- B3:  Nhấc mìn ra khỏi hố (chỉ được cầm vào thành mìn). (1,0đ)
-- B4:  Vặn nắp bảo vệ bên kíp lấy kíp ra khỏi mìn. (2,0đ)
-- B5:  Tháo ngòi nổ ra khỏi mìn. (1,0đ)
-- B6:  Thu dọn, xoá dấu vết chuyển mìn về nơi quy định. (1,0 đ)</t>
-  </si>
-  <si>
-    <t>Có 11 quy tắc an toàn khi bố trí mìn (1,0đ)
-Các quy tắc 1, 2, 3, 4, 5
-- Mọi người trong phân đội bố trí mìn phải có hiểu biết đầy đủ về cấu tạo, nguyên lý, phương pháp bố trí mìn và quy tắc bảo đảm an toàn. (2,0đ)
-- Trước khi bố trí mìn phải kiểm tra chất lượng ngòi nổ và mìn. Chỉ bố trí những quả mìn chất lượng tốt đồng bộ. (2,0đ)
-- Khi lắp ngòi nổ vào mìn phải kiểm tra lỗ lắp ngòi nổ có sạch không, có vừa không. Không được dùng sức để ấn, đập lên ngòi nổ. (2,0đ)
-- Những quả mìn đã lắp ngòi nổ cấm lăn, vứt, ném, xếp đống hoặc chồng lên nhau. (2,0đ)
-- Không mang lửa, đốt lửa nơi bố trí mìn. (1,0đ)</t>
+- Xác định hướng địch, kiểm tra chất đất, xác định vị trí bố trí mìn. (0,5đ)
+- Trải mảnh bao đựng đất và kê chân. Ngồi theo tư thế chiến sỹ, mặt quay về hướng địch. (0,5đ)
+- B1: Lấy lớp cỏ nguỵ trang dầy 3÷5 cm, rộng (60 x 60) cm, chia làm 3 mảnh, mảnh phí trước hất về hướng địch, hai mảnh quay sang hai bên; những nơi không có cỏ thì lấy lớp đất trên mặt để gọn một góc mảnh bao sau khi bố trí mìn xong tiến hành ngụy trang. (2,0đ)
+- B2: Đặt mìn ¬ướm thử đào hố. (2,0đ)
+- B3: Kiểm tra mìn, ngòi nổ. (1,0đ)
+- B4: Lắp kíp vào thân ngòi nổ, lắp ngòi nổ vào mìn. (1,0đ)
+- B5: Đặt mìn xuống hố, bố trí bẫy nếu có, rút kẹp an toàn, ấn núm khoá hết cỡ. (1,0đ)
+- B6: Lấp đất nguỵ trang, thu dọn, xoá dấu vết rời khỏi nơi bố trí. (1,0đ)</t>
+  </si>
+  <si>
+    <t>Khái niệm, nội dung trạng thái SSCĐ thường xuyên 
+a) Khái niệm (3,0đ)
+Trạng thái SSCĐ thường xuyên là bộ đội và phư¬ơng tiện kỹ thuật, VKTB ở trạng thái khi đất n¬ước thời bình, các đơn vị bộ đội tiến hành huấn luyện và SSCĐ theo kế hoạch, thời gian thống nhất. Mọi hoạt động theo chế độ XD chính quy, từng ng¬ười làm việc theo chức trách. VKTB và các phương tiện có một phần làm nhiệm vụ thường trực SSCĐ. Số còn lại cơ bản đ¬ược niêm cất bảo quản, bảo dư¬ỡng theo định kỳ. Đồng thời kế hoạch, ph¬ương án chuyển lên trạng thái SSCĐ cao hơn phải được hoàn chỉnh, hoàn thiện. 
+b) Nội dung (7,0đ)
+- Các đơn vị bộ đội công tác, hoạt động bình th¬ường theo kế hoạch tuần, tháng. (1,0đ)
+- Duy trì nghiêm túc chế độ canh, trực: Trực ban, trực chiến, trực chỉ huy. (2,0đ) 
+        + Đơn vị đủ quân làm nhiệm vụ SSCĐ duy trì 1/3 lực l¬ượng trực chiến. (0,5đ)
+        + Đơn vị pháo phòng không, súng máy phòng không đủ quân duy trì 1/3 lực lư¬ợng trực chiến. (0,5đ)
+        + Tác chiến điện tử: 1/4 lực lư¬ợng trực chiến. (0,5đ)
+        + Các đơn vị còn lại duy trì 1/9 lực l¬ượng trực chiến. 0,5đ)
+- Phương tiện, trang bị, vũ khí ngoài số quy định cho nhiệm vụ huấn luyện, canh gác, trực chiến (do cấp trên quy định) còn lại đ¬ược niêm cất, bảo quản, bảo dưỡng định kỳ theo quy định từng loại. (2,0đ)
+ - Hoàn chỉnh, hoàn thiện kế hoạch tác chiến tại chỗ, kế hoạch chống gây rối, bạo loạn và phương án chống cháy nổ. Sẵn sàng thực hiện các biện pháp chuyển trạng thái SSCĐ. (2,0đ)</t>
+  </si>
+  <si>
+    <t>Dạng câu hỏi</t>
   </si>
 </sst>
 </file>
@@ -116,13 +122,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -150,13 +157,13 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -494,51 +501,67 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3899B22-3E0E-41D7-9CED-0CAC8497C7C4}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.21875" customWidth="1"/>
     <col min="2" max="2" width="71.33203125" customWidth="1"/>
+    <col min="3" max="3" width="11.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" ht="83.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:3" ht="331.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="345.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="235.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="4" t="s">
+    <row r="4" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
     </row>
-    <row r="4" spans="1:2" ht="144" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="187.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>8</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>